<commit_message>
docs: sync design notebook with main_design.py; add design.md notes
- Rebuild notebooks/xslope_design.ipynb to mirror main_design.py: both design
  modes (fs / reliability), polygon-based rebuild_geometry (fixes the stale-
  weight bug from the old build_ground_surface path), Bishop default, run_search
  / evaluate helpers, and mode-aware verification plots.
- design.md: add a prominent admonition that this is an illustration of the
  capability (not a turnkey tool) and that custom driver code is expected and
  easy to build with agentic programming.
- design.md: note that the driver ships in the repo root as main_design.py
  (with a GitHub link) and that the Colab notebook mirrors it; give both run
  options (python main_design.py or the notebook).
- Commit the xslope_acads_simple.xlsx sample (with strength stddevs) that the
  doc links to and describes, so the download matches the text.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_acads_simple.xlsx
+++ b/docs/lem/files/xslope_acads_simple.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3293A3-B1F8-4840-BCCF-D44260C5241D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EF2E34-D733-5B43-BA55-58EC7C920AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <definedName name="solution2">mat!#REF!</definedName>
     <definedName name="version">main!$D$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="182">
   <si>
     <t>X</t>
   </si>
@@ -752,6 +752,9 @@
   </si>
   <si>
     <t>Fixity</t>
+  </si>
+  <si>
+    <t>Soil</t>
   </si>
 </sst>
 </file>
@@ -1209,13 +1212,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1392,6 +1395,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>90</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1401,6 +1416,18 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -12430,37 +12457,40 @@
       <c r="A9" s="3">
         <v>1</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Soil</t>
-        </is>
+      <c r="B9" s="3" t="s">
+        <v>181</v>
       </c>
       <c r="C9" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>mc</t>
-        </is>
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="E9" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="3">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
+      <c r="K9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L9" s="3">
+        <f>C9*0.06</f>
+        <v>1.2</v>
+      </c>
+      <c r="M9" s="3">
+        <f>E9*0.6</f>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="N9" s="3">
+        <f>F9*0.14</f>
+        <v>2.7440000000000007</v>
+      </c>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
@@ -13226,74 +13256,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="50"/>
+      <c r="D4" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="50"/>
+      <c r="G4" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="50"/>
+      <c r="J4" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="50"/>
+      <c r="M4" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="50"/>
+      <c r="P4" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="50"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="50"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="50"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="50"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="50"/>
+      <c r="AE4" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="50"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="50"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="50"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="50"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="50"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -13396,89 +13426,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="str">
+      <c r="A6" s="51" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
-      </c>
-      <c r="B6" s="51"/>
-      <c r="D6" s="50" t="str">
+        <v>Soil</v>
+      </c>
+      <c r="B6" s="52"/>
+      <c r="D6" s="51" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="51"/>
-      <c r="G6" s="50" t="str">
+      <c r="E6" s="52"/>
+      <c r="G6" s="51" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="51"/>
-      <c r="J6" s="50" t="str">
+      <c r="H6" s="52"/>
+      <c r="J6" s="51" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="51"/>
-      <c r="M6" s="50" t="str">
+      <c r="K6" s="52"/>
+      <c r="M6" s="51" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="51"/>
-      <c r="P6" s="50" t="str">
+      <c r="N6" s="52"/>
+      <c r="P6" s="51" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="51"/>
+      <c r="Q6" s="52"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="50" t="str">
+      <c r="S6" s="51" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="51"/>
+      <c r="T6" s="52"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="50" t="str">
+      <c r="V6" s="51" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="51"/>
+      <c r="W6" s="52"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="50" t="str">
+      <c r="Y6" s="51" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="51"/>
+      <c r="Z6" s="52"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="50" t="str">
+      <c r="AB6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="51"/>
-      <c r="AE6" s="50" t="str">
+      <c r="AC6" s="52"/>
+      <c r="AE6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="51"/>
+      <c r="AF6" s="52"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="50" t="str">
+      <c r="AH6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="51"/>
+      <c r="AI6" s="52"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="50" t="str">
+      <c r="AK6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="51"/>
+      <c r="AL6" s="52"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="50" t="str">
+      <c r="AN6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="51"/>
+      <c r="AO6" s="52"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="50" t="str">
+      <c r="AQ6" s="51" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="51"/>
+      <c r="AR6" s="52"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -13582,7 +13612,7 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B8" s="3">
         <v>25</v>
@@ -13714,7 +13744,7 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="B11" s="3">
         <v>35</v>
@@ -14398,36 +14428,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14465,74 +14495,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="50" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="50"/>
+      <c r="D4" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="50"/>
+      <c r="G4" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="50"/>
+      <c r="J4" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="50"/>
+      <c r="M4" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="50"/>
+      <c r="P4" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="50"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="50"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="50"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="50"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="50"/>
+      <c r="AE4" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="50"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="50" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="50"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="50"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="50"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="50"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -14637,7 +14667,7 @@
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>Soil</v>
       </c>
       <c r="B6" s="54"/>
       <c r="D6" s="53" t="str">
@@ -15621,12 +15651,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -15643,14 +15675,12 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15873,10 +15903,8 @@
       <c r="C3" s="3">
         <v>45</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
+      <c r="D3" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3">
@@ -15903,10 +15931,8 @@
       <c r="C4" s="3">
         <v>48</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Depth</t>
-        </is>
+      <c r="D4" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="E4" s="3">
         <v>20</v>

</xml_diff>

<commit_message>
fix(models): every sample model wears the template's rich headers — γsat, σ(·), θp
The mangled-template era left plain-ASCII copies of the template's seven
rich-text header cells (mat γsat + the five σ() standard-deviation headers,
piles θp) in all 39 sample models and vp049 — the piles sheet render was still
showing 'qp'. One-cell XML transplants of the template's own runs, data and
locked results untouched; every file still loads. lem09_sheet_piles and the
usage sheet_piles render now show θp.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_acads_simple.xlsx
+++ b/docs/lem/files/xslope_acads_simple.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="318">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -992,6 +992,167 @@
   </si>
   <si>
     <t>auto</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>g</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(c)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(c/p)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(d)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>s(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>psi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>g</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>sat</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>q</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3243,7 +3404,7 @@
         <v>270</v>
       </c>
       <c r="H2" s="40" t="s">
-        <v>271</v>
+        <v>317</v>
       </c>
       <c r="I2" s="40" t="s">
         <v>253</v>
@@ -5722,7 +5883,7 @@
         <v>111</v>
       </c>
       <c r="D10" s="48" t="s">
-        <v>112</v>
+        <v>316</v>
       </c>
       <c r="E10" s="44" t="s">
         <v>113</v>
@@ -5791,22 +5952,22 @@
         <v>133</v>
       </c>
       <c r="AA10" s="46" t="s">
-        <v>134</v>
+        <v>311</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>135</v>
+        <v>312</v>
       </c>
       <c r="AC10" s="47" t="s">
         <v>136</v>
       </c>
       <c r="AD10" s="46" t="s">
-        <v>137</v>
+        <v>313</v>
       </c>
       <c r="AE10" s="46" t="s">
-        <v>138</v>
+        <v>314</v>
       </c>
       <c r="AF10" s="47" t="s">
-        <v>139</v>
+        <v>315</v>
       </c>
       <c r="AG10" s="23" t="s">
         <v>140</v>

</xml_diff>